<commit_message>
passage au thème + makefile
</commit_message>
<xml_diff>
--- a/template/horaire-rencontres.xlsx
+++ b/template/horaire-rencontres.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/etiennerivard/notes_de_cours/projetpersonnel/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5760F22-F040-DC4A-A674-1ED9771CE3B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AEA48A8-C49E-E842-94DE-DC06668A9550}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3000" yWindow="1580" windowWidth="27080" windowHeight="16440" xr2:uid="{4696F4E7-E751-AB46-8D30-A385E7EE1466}"/>
   </bookViews>
   <sheets>
-    <sheet name="rencontre-fin" sheetId="2" r:id="rId1"/>
+    <sheet name="horaire" sheetId="2" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="ListeEtudiants_cours4206C3VI_gr00001" localSheetId="0">'rencontre-fin'!$B$1:$D$20</definedName>
+    <definedName name="ListeEtudiants_cours4206C3VI_gr00001" localSheetId="0">horaire!$B$1:$D$20</definedName>
     <definedName name="temps_rencontre">Sheet2!$A$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>

</xml_diff>

<commit_message>
changement horaire jour 2
</commit_message>
<xml_diff>
--- a/template/horaire-rencontres.xlsx
+++ b/template/horaire-rencontres.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/etiennerivard/notes_de_cours/projetpersonnel/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA09EAE-CF91-8248-8EEC-B3C696785F5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ED9F05A-A47B-EB42-8909-A050AA136564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3000" yWindow="1580" windowWidth="27080" windowHeight="16440" xr2:uid="{4696F4E7-E751-AB46-8D30-A385E7EE1466}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="ListeEtudiants_cours4206C3VI_gr00001" localSheetId="0">horaire!$B$1:$C$20</definedName>
+    <definedName name="ListeEtudiants_cours4206C3VI_gr00001" localSheetId="0">horaire!$B$1:$C$5</definedName>
     <definedName name="temps_rencontre">Sheet2!$A$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Nom de l'étudiant</t>
   </si>
@@ -64,55 +64,10 @@
     <t>Date et heure</t>
   </si>
   <si>
-    <t>Yohan R.</t>
-  </si>
-  <si>
-    <t>Morgan B.</t>
-  </si>
-  <si>
-    <t>Anthony R.</t>
-  </si>
-  <si>
-    <t>Nathan G.</t>
-  </si>
-  <si>
-    <t>Philippe-Vu B.</t>
-  </si>
-  <si>
-    <t>Félix D.</t>
-  </si>
-  <si>
-    <t>Hugo N.</t>
-  </si>
-  <si>
-    <t>Achraf E.</t>
-  </si>
-  <si>
-    <t>Rachid T.</t>
-  </si>
-  <si>
-    <t>Bady Pascal F.</t>
-  </si>
-  <si>
-    <t>Breno G.</t>
-  </si>
-  <si>
     <t>Derek B.</t>
   </si>
   <si>
-    <t>William C.</t>
-  </si>
-  <si>
     <t>Justin C.</t>
-  </si>
-  <si>
-    <t>Leandre Junior K.</t>
-  </si>
-  <si>
-    <t>Frédérick B.</t>
-  </si>
-  <si>
-    <t>Nathan R.</t>
   </si>
   <si>
     <t>Zacharie N.</t>
@@ -486,7 +441,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B272E60-778B-BE4F-ACE9-8294C423DABC}">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.5" bestFit="1" customWidth="1"/>
@@ -503,7 +458,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
-        <v>46239.541666666664</v>
+        <v>46240.375</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
@@ -511,8 +466,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
-        <f t="shared" ref="A3:A13" si="0">A2+temps_rencontre</f>
-        <v>46239.552083333328</v>
+        <v>46240.385416666664</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
@@ -520,8 +474,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
-        <f t="shared" si="0"/>
-        <v>46239.562499999993</v>
+        <v>46240.395833333328</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
@@ -529,145 +482,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
-        <f t="shared" si="0"/>
-        <v>46239.572916666657</v>
+        <v>46240.406249999993</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="2">
-        <f t="shared" si="0"/>
-        <v>46239.583333333321</v>
-      </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
-        <f t="shared" si="0"/>
-        <v>46239.593749999985</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="2">
-        <f t="shared" si="0"/>
-        <v>46239.60416666665</v>
-      </c>
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="2">
-        <f t="shared" si="0"/>
-        <v>46239.614583333314</v>
-      </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="2">
-        <f t="shared" si="0"/>
-        <v>46239.624999999978</v>
-      </c>
-      <c r="B10" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="2">
-        <f t="shared" si="0"/>
-        <v>46239.635416666642</v>
-      </c>
-      <c r="B11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="2">
-        <f t="shared" si="0"/>
-        <v>46239.645833333307</v>
-      </c>
-      <c r="B12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="2">
-        <f t="shared" si="0"/>
-        <v>46239.656249999971</v>
-      </c>
-      <c r="B13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>46240.375</v>
-      </c>
-      <c r="B14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" s="2">
-        <f t="shared" ref="A15:A20" si="1">A14+temps_rencontre</f>
-        <v>46240.385416666664</v>
-      </c>
-      <c r="B15" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="2">
-        <f t="shared" si="1"/>
-        <v>46240.395833333328</v>
-      </c>
-      <c r="B16" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="2">
-        <f t="shared" si="1"/>
-        <v>46240.406249999993</v>
-      </c>
-      <c r="B17" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="2">
-        <f t="shared" si="1"/>
-        <v>46240.416666666657</v>
-      </c>
-      <c r="B18" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="2">
-        <f t="shared" si="1"/>
-        <v>46240.427083333321</v>
-      </c>
-      <c r="B19" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="2">
-        <f t="shared" si="1"/>
-        <v>46240.437499999985</v>
-      </c>
-      <c r="B20" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>